<commit_message>
[FE,BE]: Download file with progress bar demo
</commit_message>
<xml_diff>
--- a/extra/springboot-template/input/test.xlsx
+++ b/extra/springboot-template/input/test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\CODING\java-is-fun\extra\springboot-template\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9A39A87-E0F0-43C7-82C8-D462E2B959B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12327C9C-1273-4509-9E56-50A1E8E624C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="35580" yWindow="3735" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -51,7 +51,7 @@
     <t>Red me</t>
   </si>
   <si>
-    <t>{{my_name}}</t>
+    <t>{{my_name2}}</t>
   </si>
 </sst>
 </file>

</xml_diff>